<commit_message>
Fix GL 8121 VTTB VAT transfer matching for pair 1363111-3363111
</commit_message>
<xml_diff>
--- a/đầu ra/Bao_Cao_Doi_Soat_136_336_Thang_7_2026.xlsx
+++ b/đầu ra/Bao_Cao_Doi_Soat_136_336_Thang_7_2026.xlsx
@@ -1947,7 +1947,7 @@
       </c>
       <c r="F8" s="16" t="inlineStr">
         <is>
-          <t>🏢 Bút Toán Điện Lực Bị Thiếu (1 chứng từ)</t>
+          <t>🏢 Bút Toán Điện Lực Bị Thiếu (0 chứng từ)</t>
         </is>
       </c>
     </row>
@@ -2014,24 +2014,14 @@
         </is>
       </c>
       <c r="E10" t="inlineStr"/>
-      <c r="F10" s="18" t="inlineStr">
-        <is>
-          <t>2026-07-31</t>
-        </is>
-      </c>
-      <c r="G10" s="18" t="inlineStr">
-        <is>
-          <t>8121</t>
-        </is>
-      </c>
-      <c r="H10" s="19" t="n">
-        <v>86064000</v>
-      </c>
-      <c r="I10" s="20" t="inlineStr">
-        <is>
-          <t>KC thuế GTGT điều động tháng 7/2026 sang công nợ thuế GTGT điện</t>
-        </is>
-      </c>
+      <c r="F10" s="21" t="inlineStr">
+        <is>
+          <t>✅ Phía Điện lực đã hạch toán đầy đủ.</t>
+        </is>
+      </c>
+      <c r="G10" s="22" t="n"/>
+      <c r="H10" s="22" t="n"/>
+      <c r="I10" s="22" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="18" t="inlineStr">
@@ -4372,83 +4362,84 @@
       <c r="E170" t="inlineStr"/>
     </row>
   </sheetData>
-  <mergeCells count="76">
-    <mergeCell ref="A25:I25"/>
+  <mergeCells count="77">
+    <mergeCell ref="A97:D97"/>
+    <mergeCell ref="A29:D29"/>
+    <mergeCell ref="F117:I117"/>
+    <mergeCell ref="F53:I53"/>
+    <mergeCell ref="F29:I29"/>
+    <mergeCell ref="A94:I95"/>
+    <mergeCell ref="A51:D51"/>
+    <mergeCell ref="A107:D107"/>
+    <mergeCell ref="A35:I35"/>
+    <mergeCell ref="A84:I85"/>
+    <mergeCell ref="A59:I59"/>
+    <mergeCell ref="A103:I103"/>
+    <mergeCell ref="A5:I6"/>
+    <mergeCell ref="F97:I97"/>
+    <mergeCell ref="A134:I135"/>
+    <mergeCell ref="A46:I46"/>
+    <mergeCell ref="A19:D19"/>
+    <mergeCell ref="A117:D117"/>
+    <mergeCell ref="F107:I107"/>
+    <mergeCell ref="A127:D127"/>
+    <mergeCell ref="A114:I115"/>
+    <mergeCell ref="F19:I19"/>
+    <mergeCell ref="F63:I63"/>
+    <mergeCell ref="A60:I61"/>
+    <mergeCell ref="A16:I17"/>
+    <mergeCell ref="A93:I93"/>
+    <mergeCell ref="A102:I102"/>
+    <mergeCell ref="A124:I125"/>
+    <mergeCell ref="A34:I34"/>
+    <mergeCell ref="A83:I83"/>
+    <mergeCell ref="A137:D137"/>
+    <mergeCell ref="A92:I92"/>
+    <mergeCell ref="A74:D74"/>
+    <mergeCell ref="F109:I109"/>
+    <mergeCell ref="A129:D129"/>
+    <mergeCell ref="A69:I69"/>
     <mergeCell ref="A8:D8"/>
-    <mergeCell ref="A97:D97"/>
-    <mergeCell ref="A46:I46"/>
     <mergeCell ref="A133:I133"/>
     <mergeCell ref="F39:I39"/>
     <mergeCell ref="A109:D109"/>
-    <mergeCell ref="A29:D29"/>
     <mergeCell ref="A3:I3"/>
-    <mergeCell ref="A19:D19"/>
     <mergeCell ref="A63:D63"/>
-    <mergeCell ref="F117:I117"/>
-    <mergeCell ref="A117:D117"/>
-    <mergeCell ref="F107:I107"/>
     <mergeCell ref="A113:I113"/>
-    <mergeCell ref="A47:I47"/>
-    <mergeCell ref="F53:I53"/>
-    <mergeCell ref="A127:D127"/>
-    <mergeCell ref="A114:I115"/>
     <mergeCell ref="A14:I14"/>
     <mergeCell ref="A39:D39"/>
     <mergeCell ref="A48:I49"/>
     <mergeCell ref="F87:I87"/>
-    <mergeCell ref="F29:I29"/>
-    <mergeCell ref="A94:I95"/>
+    <mergeCell ref="A4:I4"/>
+    <mergeCell ref="F10:I10"/>
+    <mergeCell ref="F137:I137"/>
+    <mergeCell ref="F89:I89"/>
+    <mergeCell ref="F74:I74"/>
+    <mergeCell ref="A87:D87"/>
+    <mergeCell ref="F139:I139"/>
+    <mergeCell ref="A65:D65"/>
+    <mergeCell ref="A71:I72"/>
+    <mergeCell ref="A24:I24"/>
+    <mergeCell ref="F76:I76"/>
+    <mergeCell ref="A82:I82"/>
+    <mergeCell ref="F8:I8"/>
+    <mergeCell ref="A123:I123"/>
+    <mergeCell ref="A132:I132"/>
+    <mergeCell ref="A25:I25"/>
+    <mergeCell ref="A47:I47"/>
     <mergeCell ref="A122:I122"/>
-    <mergeCell ref="A51:D51"/>
-    <mergeCell ref="F19:I19"/>
-    <mergeCell ref="A35:I35"/>
-    <mergeCell ref="A4:I4"/>
-    <mergeCell ref="F63:I63"/>
-    <mergeCell ref="A84:I85"/>
-    <mergeCell ref="A107:D107"/>
-    <mergeCell ref="A60:I61"/>
-    <mergeCell ref="F137:I137"/>
     <mergeCell ref="A36:I37"/>
-    <mergeCell ref="A16:I17"/>
-    <mergeCell ref="F89:I89"/>
     <mergeCell ref="A112:I112"/>
     <mergeCell ref="F127:I127"/>
     <mergeCell ref="A119:D119"/>
-    <mergeCell ref="A93:I93"/>
-    <mergeCell ref="F74:I74"/>
-    <mergeCell ref="A102:I102"/>
-    <mergeCell ref="A124:I125"/>
-    <mergeCell ref="A87:D87"/>
-    <mergeCell ref="F139:I139"/>
     <mergeCell ref="F21:I21"/>
-    <mergeCell ref="A65:D65"/>
     <mergeCell ref="A58:I58"/>
-    <mergeCell ref="A71:I72"/>
-    <mergeCell ref="A34:I34"/>
     <mergeCell ref="F51:I51"/>
-    <mergeCell ref="A83:I83"/>
-    <mergeCell ref="A137:D137"/>
-    <mergeCell ref="A92:I92"/>
-    <mergeCell ref="A24:I24"/>
     <mergeCell ref="A26:I27"/>
     <mergeCell ref="A15:I15"/>
-    <mergeCell ref="A59:I59"/>
-    <mergeCell ref="F76:I76"/>
-    <mergeCell ref="A82:I82"/>
-    <mergeCell ref="A74:D74"/>
-    <mergeCell ref="A103:I103"/>
-    <mergeCell ref="F8:I8"/>
-    <mergeCell ref="A5:I6"/>
-    <mergeCell ref="F97:I97"/>
-    <mergeCell ref="F109:I109"/>
-    <mergeCell ref="A123:I123"/>
     <mergeCell ref="F129:I129"/>
-    <mergeCell ref="A132:I132"/>
     <mergeCell ref="A70:I70"/>
-    <mergeCell ref="A134:I135"/>
     <mergeCell ref="A104:I105"/>
-    <mergeCell ref="A129:D129"/>
-    <mergeCell ref="A69:I69"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>